<commit_message>
Move the secretariat on the sketch; add the 27-30 October banner mock-up
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/動態表_ACDR2026_as_of_25_Sep_v2_9.xlsx
+++ b/reports/acdr2026_staff_deployment/動態表_ACDR2026_as_of_25_Sep_v2_9.xlsx
@@ -1184,49 +1184,31 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
+  <oneCellAnchor>
     <from>
       <col>0</col>
       <colOff>0</colOff>
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <to>
-      <col>18</col>
-      <colOff>540262</colOff>
-      <row>26</row>
-      <rowOff>142875</rowOff>
-    </to>
+    <ext cx="15116175" cy="6438900"/>
     <pic>
       <nvPicPr>
-        <cNvPr id="3" name="図 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="11562048" cy="4918982"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
-  </twoCellAnchor>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1275,6 +1257,31 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9525000" cy="2514600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -6167,7 +6174,9 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1"/>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -6179,13 +6188,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="H15:H15"/>
+  <dimension ref="A15:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="15">
       <c r="H15" s="160" t="inlineStr">
         <is>
           <t>２７－３０</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ADRC 修正案モックアップ（9/25）: 27-30 October 2026 と Singapore Expo を1行に</t>
         </is>
       </c>
     </row>
@@ -11026,8 +11042,8 @@
     <mergeCell ref="M11:U11"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="Y11:AD11"/>
+    <mergeCell ref="N4:U4"/>
     <mergeCell ref="M10:U10"/>
-    <mergeCell ref="N4:U4"/>
     <mergeCell ref="D27:F27"/>
     <mergeCell ref="Y14:AD14"/>
     <mergeCell ref="G4:J4"/>
@@ -12069,7 +12085,6 @@
     <row r="2" ht="31.5" customHeight="1" s="89">
       <c r="A2" s="88" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="89">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -12516,7 +12531,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="89">
       <c r="A4" s="70" t="inlineStr">
         <is>
@@ -14805,7 +14819,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58">
       <c r="B58" s="77" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Sketch: 8-seat ADRC secretariat block in the upper left, left side row reduced to 8
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/動態表_ACDR2026_as_of_25_Sep_v2_9.xlsx
+++ b/reports/acdr2026_staff_deployment/動態表_ACDR2026_as_of_25_Sep_v2_9.xlsx
@@ -1235,7 +1235,7 @@
         </cNvPicPr>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
         <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
@@ -1271,13 +1271,16 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6174,9 +6177,7 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <sheetData>
-    <row r="1"/>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
@@ -11042,8 +11043,8 @@
     <mergeCell ref="M11:U11"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="Y11:AD11"/>
+    <mergeCell ref="M10:U10"/>
     <mergeCell ref="N4:U4"/>
-    <mergeCell ref="M10:U10"/>
     <mergeCell ref="D27:F27"/>
     <mergeCell ref="Y14:AD14"/>
     <mergeCell ref="G4:J4"/>

</xml_diff>